<commit_message>
ya me falta la elección de grados en el acta de inicio
</commit_message>
<xml_diff>
--- a/3_documentos_actas/parejas_practica_v.xlsx
+++ b/3_documentos_actas/parejas_practica_v.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marco\Documentos\docencia\practica_v_dllo_pto_math_infancia\3_documentos_actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F20067A0-C170-45C6-B8D6-41AD6F8EDF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CFEB085-B7EF-43D0-B20E-F459273A1300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,77 +33,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
-  <si>
-    <t>Grado 3</t>
-  </si>
-  <si>
-    <t>Grado_7</t>
-  </si>
-  <si>
-    <t>Groado_8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingrid González </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eliana Arrieta, </t>
-  </si>
-  <si>
-    <t>¥ Katherine Quiroz</t>
-  </si>
-  <si>
-    <t>Grado: 3°</t>
-  </si>
-  <si>
-    <t>Jenifer Rivera. Grado 3A</t>
-  </si>
-  <si>
-    <t>Danna</t>
-  </si>
-  <si>
-    <t>Grupo_9</t>
-  </si>
-  <si>
-    <t>Grupo_10</t>
-  </si>
-  <si>
-    <t>Dayana</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Preescolar</t>
   </si>
   <si>
-    <t>Cedulas</t>
-  </si>
-  <si>
-    <t>GrupoPracticantes</t>
-  </si>
-  <si>
-    <t>Emails</t>
-  </si>
-  <si>
     <t>Grado</t>
   </si>
   <si>
-    <t>Salon</t>
-  </si>
-  <si>
-    <t>ItemGrupo</t>
-  </si>
-  <si>
     <t>Ítem</t>
   </si>
   <si>
     <t>Nombres</t>
   </si>
   <si>
-    <t>['Alvarez Perez Carlos Julio', 'Sara Guerra']</t>
-  </si>
-  <si>
-    <t>["Yesika Martinez", "Xiomara López"]</t>
-  </si>
-  <si>
     <t>grupo_2</t>
   </si>
   <si>
@@ -141,13 +84,34 @@
   </si>
   <si>
     <t>grupo_7</t>
+  </si>
+  <si>
+    <t>grupo_8</t>
+  </si>
+  <si>
+    <t>grupo_9</t>
+  </si>
+  <si>
+    <t>grupo_10</t>
+  </si>
+  <si>
+    <t>['Ingrid Gonzalez', 'Katherine Quiroz']</t>
+  </si>
+  <si>
+    <t>['Eliana Arrieta', 'Jenifer Rivera']</t>
+  </si>
+  <si>
+    <t>['Danna', '']</t>
+  </si>
+  <si>
+    <t>['Dayana', '']</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,14 +141,6 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -209,16 +165,16 @@
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -494,244 +450,133 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
     <col min="2" max="2" width="38.6640625" customWidth="1"/>
-    <col min="3" max="3" width="36.44140625" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
-    <col min="5" max="5" width="16.109375" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
         <v>19</v>
       </c>
-      <c r="B1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+      <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="4"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="7"/>
-      <c r="C10" s="4"/>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="7"/>
-      <c r="C11" s="4"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="D13" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>2</v>
-      </c>
-      <c r="F13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G13" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="D14" t="s">
-        <v>3</v>
-      </c>
-      <c r="E14" t="s">
-        <v>4</v>
-      </c>
-      <c r="F14" t="s">
-        <v>8</v>
-      </c>
-      <c r="G14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="D15" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" t="s">
-        <v>7</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="C11" s="5" t="s">
         <v>0</v>
-      </c>
-      <c r="G15" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="D16" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" t="s">
-        <v>13</v>
-      </c>
-      <c r="E18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19">
-        <v>1</v>
-      </c>
-      <c r="C19" t="s">
-        <v>22</v>
-      </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20">
-        <v>2</v>
-      </c>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21">
-        <v>3</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" s="4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29">
-        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>